<commit_message>
chore: add debug logs and adjust some code
1. add request params log in getProjects api
2. remove useless slog comment in employees handler
3. adjust getProjects call with page size param and add response log
4. add project name passing in menu navigation
5. comment out total column code in attendance page
</commit_message>
<xml_diff>
--- a/测试数据20260603/测试数据20260603/固定信息表-Employee fixed data template20260603.xlsx
+++ b/测试数据20260603/测试数据20260603/固定信息表-Employee fixed data template20260603.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\e16\code\react\kairis-gw\测试数据20260603\测试数据20260603\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10E0CC8A-181D-4FA9-AF39-99950DA5F882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B25FECE7-F113-406B-96F6-49E2FE237FD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6B964242-7783-4F55-9B37-964571950F25}"/>
   </bookViews>
@@ -150,78 +150,77 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
+    <t>abc</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>aabbcc</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>dflj.jlkjl</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3456789012</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>jkjlen,.jlsdfj.jljl</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>4567890123</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TK/0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Office Boy</t>
+  </si>
+  <si>
+    <t>K/2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IT &amp; Business Development</t>
+  </si>
+  <si>
+    <t>K/3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>HRD Supervisor</t>
+  </si>
+  <si>
+    <t>TK/3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Finance Senior Officer</t>
+  </si>
+  <si>
+    <t>Post_Function_alw/Month</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Accommodation_alw/Month</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>test@gdap-indo.com</t>
+  </si>
+  <si>
     <t>Head Office Jakarta</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>abc</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>aabbcc</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>dflj.jlkjl</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>3456789012</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>jkjlen,.jlsdfj.jljl</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>4567890123</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>TK/0</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Office Boy</t>
-  </si>
-  <si>
-    <t>K/2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>IT &amp; Business Development</t>
-  </si>
-  <si>
-    <t>K/3</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>HRD Supervisor</t>
-  </si>
-  <si>
-    <t>TK/3</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Finance Senior Officer</t>
-  </si>
-  <si>
-    <t>Post_Function_alw/Month</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Accommodation_alw/Month</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>test@gdap-indo.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -289,6 +288,12 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -336,7 +341,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -390,6 +395,9 @@
     </xf>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -773,7 +781,7 @@
         <v>6</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N1" s="4" t="s">
         <v>7</v>
@@ -800,7 +808,7 @@
         <v>14</v>
       </c>
       <c r="V1" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="W1" s="4" t="s">
         <v>15</v>
@@ -827,27 +835,27 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:30" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A2" s="6">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>28</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>29</v>
       </c>
       <c r="D2" s="8">
         <v>1234567890</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F2" s="7">
         <v>0</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H2" s="13">
         <v>45444</v>
@@ -859,7 +867,7 @@
         <v>23870</v>
       </c>
       <c r="K2" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="L2" s="16">
         <v>5000000</v>
@@ -923,23 +931,23 @@
       <c r="A3" s="6">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="s">
-        <v>28</v>
+      <c r="B3" s="18" t="s">
+        <v>45</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D3" s="10">
         <v>2345678901</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F3" s="12">
         <v>0.01</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H3" s="15">
         <v>44682</v>
@@ -951,7 +959,7 @@
         <v>29709</v>
       </c>
       <c r="K3" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="L3" s="17">
         <v>7000000</v>
@@ -1011,27 +1019,27 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:30" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A4" s="6">
         <v>3</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>28</v>
+      <c r="B4" s="18" t="s">
+        <v>45</v>
       </c>
       <c r="C4" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="10" t="s">
-        <v>32</v>
-      </c>
       <c r="E4" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F4" s="12">
         <v>0.04</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H4" s="15">
         <v>45842</v>
@@ -1043,7 +1051,7 @@
         <v>33820</v>
       </c>
       <c r="K4" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="L4" s="17">
         <v>10000000</v>
@@ -1107,23 +1115,23 @@
       <c r="A5" s="6">
         <v>4</v>
       </c>
-      <c r="B5" s="7" t="s">
-        <v>28</v>
+      <c r="B5" s="18" t="s">
+        <v>45</v>
       </c>
       <c r="C5" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>34</v>
-      </c>
       <c r="E5" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F5" s="12">
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H5" s="15">
         <v>46174</v>
@@ -1135,7 +1143,7 @@
         <v>23704</v>
       </c>
       <c r="K5" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="L5" s="17">
         <v>20000000</v>

</xml_diff>